<commit_message>
Agregada automatización de noticias con IA
</commit_message>
<xml_diff>
--- a/links/Juegos_PC.xlsx
+++ b/links/Juegos_PC.xlsx
@@ -397,14 +397,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P21"/>
+  <dimension ref="A1:Q21"/>
   <cols>
     <col min="1" max="1" width="45.83203125" customWidth="1"/>
     <col min="2" max="2" width="45.83203125" customWidth="1"/>
     <col min="3" max="3" width="45.83203125" customWidth="1"/>
     <col min="4" max="4" width="30.83203125" customWidth="1"/>
-    <col min="5" max="5" width="20.83203125" customWidth="1"/>
-    <col min="6" max="6" width="35.83203125" customWidth="1"/>
+    <col min="5" max="5" width="50.83203125" customWidth="1"/>
+    <col min="6" max="6" width="20.83203125" customWidth="1"/>
     <col min="7" max="7" width="35.83203125" customWidth="1"/>
     <col min="8" max="8" width="35.83203125" customWidth="1"/>
     <col min="9" max="9" width="35.83203125" customWidth="1"/>
@@ -415,6 +415,7 @@
     <col min="14" max="14" width="35.83203125" customWidth="1"/>
     <col min="15" max="15" width="35.83203125" customWidth="1"/>
     <col min="16" max="16" width="35.83203125" customWidth="1"/>
+    <col min="17" max="17" width="35.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -431,39 +432,42 @@
         <v>Imagen Local</v>
       </c>
       <c r="E1" t="str">
+        <v>Sinopsis</v>
+      </c>
+      <c r="F1" t="str">
         <v>En Varias Partes</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Mega</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Mediafire</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>1Fichier</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Google Drive</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>Qiwi</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>Pixeldrain</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>Megaup</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>Otro Link 1</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>Otro Link 2</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
         <v>Otro Link 3</v>
       </c>
-      <c r="P1" t="str">
+      <c r="Q1" t="str">
         <v>Otro Link 4</v>
       </c>
     </row>
@@ -481,21 +485,24 @@
         <v>imagenes/PC/Killer Bean.jpg</v>
       </c>
       <c r="E2" t="str">
-        <v>No</v>
-      </c>
-      <c r="H2" t="str">
+        <v>No disponible</v>
+      </c>
+      <c r="F2" t="str">
+        <v>No</v>
+      </c>
+      <c r="I2" t="str">
         <v>https://1fichier.com/?925i8nko0scdqavz9dwm</v>
       </c>
-      <c r="L2" t="str">
+      <c r="M2" t="str">
         <v>https://megaup.net/26dbdefb5b2d7d44e48646cfb1b970d6/Killer.Bean.rar</v>
       </c>
-      <c r="M2" t="str">
+      <c r="N2" t="str">
         <v>https://bowfile.com/2982G</v>
       </c>
-      <c r="N2" t="str">
+      <c r="O2" t="str">
         <v>https://gofile.io/d/bJ5SFe</v>
       </c>
-      <c r="O2" t="str">
+      <c r="P2" t="str">
         <v>https://downloadgameps3.net/archives/18667</v>
       </c>
     </row>
@@ -513,24 +520,27 @@
         <v>imagenes/PC/Arms of God.jpg</v>
       </c>
       <c r="E3" t="str">
-        <v>No</v>
+        <v>No disponible</v>
       </c>
       <c r="F3" t="str">
+        <v>No</v>
+      </c>
+      <c r="G3" t="str">
         <v>https://mega.nz/file/Ol5jVRTZ#oMg3KKox5uvhDzKbTlbKiXc6PNjVY4jLb6ecjnjmoxE</v>
       </c>
-      <c r="H3" t="str">
+      <c r="I3" t="str">
         <v>https://1fichier.com/?oyfsnbcsfl2fmn6gtlo7</v>
       </c>
-      <c r="L3" t="str">
+      <c r="M3" t="str">
         <v>https://megaup.net/55818b38fe3a2a0efacc27aca345ea3e/Arms.of.God.rar</v>
       </c>
-      <c r="M3" t="str">
+      <c r="N3" t="str">
         <v>https://send.now/7llxphba5m72</v>
       </c>
-      <c r="N3" t="str">
+      <c r="O3" t="str">
         <v>https://gofile.io/d/1uiO1Z</v>
       </c>
-      <c r="O3" t="str">
+      <c r="P3" t="str">
         <v>https://downloadgameps3.net/archives/18667</v>
       </c>
     </row>
@@ -548,24 +558,27 @@
         <v>imagenes/PC/Duppy Detective Tashia.jpg</v>
       </c>
       <c r="E4" t="str">
-        <v>No</v>
+        <v>No disponible</v>
       </c>
       <c r="F4" t="str">
+        <v>No</v>
+      </c>
+      <c r="G4" t="str">
         <v>https://mega.nz/file/BqohVaoJ#1Uph-Ez1yrU4-18jRCvV3n9rsOqo6dmANs9si0HV_XM</v>
       </c>
-      <c r="H4" t="str">
+      <c r="I4" t="str">
         <v>https://1fichier.com/?4ioj31e2s48rb8if1ibj</v>
       </c>
-      <c r="L4" t="str">
+      <c r="M4" t="str">
         <v>https://megaup.net/029a026346b8e29822915d93802e87c6/Duppy.Detective.Tashia-TENOKE.rar</v>
       </c>
-      <c r="M4" t="str">
+      <c r="N4" t="str">
         <v>https://send.now/d/1lMeA</v>
       </c>
-      <c r="N4" t="str">
+      <c r="O4" t="str">
         <v>https://gofile.io/d/4IxgSE</v>
       </c>
-      <c r="O4" t="str">
+      <c r="P4" t="str">
         <v>https://downloadgameps3.net/archives/18667</v>
       </c>
     </row>
@@ -583,24 +596,27 @@
         <v>imagenes/PC/Voidling Bound.jpg</v>
       </c>
       <c r="E5" t="str">
-        <v>No</v>
+        <v>No disponible</v>
       </c>
       <c r="F5" t="str">
+        <v>No</v>
+      </c>
+      <c r="G5" t="str">
         <v>https://mega.nz/file/QFUCSL4a#1O-TFGfr0G6LwR636n-mLir8x-hZ_fF24XBH_2cDPrs</v>
       </c>
-      <c r="H5" t="str">
+      <c r="I5" t="str">
         <v>https://1fichier.com/?xsetfxi00ddxkizpuppw</v>
       </c>
-      <c r="L5" t="str">
+      <c r="M5" t="str">
         <v>https://megaup.net/80963507d69f87e0a8a759bf5a214b57/Voidling.Bound.rar</v>
       </c>
-      <c r="M5" t="str">
+      <c r="N5" t="str">
         <v>https://bowfile.com/29846</v>
       </c>
-      <c r="N5" t="str">
+      <c r="O5" t="str">
         <v>https://gofile.io/d/3aZomE</v>
       </c>
-      <c r="O5" t="str">
+      <c r="P5" t="str">
         <v>https://downloadgameps3.net/archives/18667</v>
       </c>
     </row>
@@ -618,24 +634,27 @@
         <v>imagenes/PC/Insomnia Chapter One.jpg</v>
       </c>
       <c r="E6" t="str">
-        <v>No</v>
+        <v>No disponible</v>
       </c>
       <c r="F6" t="str">
+        <v>No</v>
+      </c>
+      <c r="G6" t="str">
         <v>https://mega.nz/file/x6JB0B5K#-CiFXfBQam9NGlww_AlyWIk7DPEov3t9yMySHNZK47g</v>
       </c>
-      <c r="H6" t="str">
+      <c r="I6" t="str">
         <v>https://1fichier.com/?vbu4d71mkzl3wrctmrbt</v>
       </c>
-      <c r="L6" t="str">
+      <c r="M6" t="str">
         <v>https://megaup.net/56918fbd98f5f0b375f11dae0c0217a4/Insomnia.Chapter.One-TENOKE.rar</v>
       </c>
-      <c r="M6" t="str">
+      <c r="N6" t="str">
         <v>https://send.now/d/1lMej</v>
       </c>
-      <c r="N6" t="str">
+      <c r="O6" t="str">
         <v>https://gofile.io/d/MqWObh</v>
       </c>
-      <c r="O6" t="str">
+      <c r="P6" t="str">
         <v>https://downloadgameps3.net/archives/18667</v>
       </c>
     </row>
@@ -653,24 +672,27 @@
         <v>imagenes/PC/MEAT 2 Absolute Zero.jpg</v>
       </c>
       <c r="E7" t="str">
-        <v>No</v>
-      </c>
-      <c r="H7" t="str">
+        <v>No disponible</v>
+      </c>
+      <c r="F7" t="str">
+        <v>No</v>
+      </c>
+      <c r="I7" t="str">
         <v>https://1fichier.com/?44hx6b6rr8ggxx1svy2p</v>
       </c>
-      <c r="L7" t="str">
+      <c r="M7" t="str">
         <v>https://megaup.net/fb26d9ef63b99fc2ff199b8bb7575af2/MEAT.2.Absolute.Zero.rar</v>
       </c>
-      <c r="M7" t="str">
+      <c r="N7" t="str">
         <v>https://bowfile.com/1tasn</v>
       </c>
-      <c r="N7" t="str">
+      <c r="O7" t="str">
         <v>https://send.now/d/1lMgY</v>
       </c>
-      <c r="O7" t="str">
+      <c r="P7" t="str">
         <v>https://gofile.io/d/GDhkbi</v>
       </c>
-      <c r="P7" t="str">
+      <c r="Q7" t="str">
         <v>https://downloadgameps3.net/archives/18667</v>
       </c>
     </row>
@@ -688,18 +710,21 @@
         <v>imagenes/PC/SubZero.jpg</v>
       </c>
       <c r="E8" t="str">
-        <v>No</v>
-      </c>
-      <c r="H8" t="str">
+        <v>No disponible</v>
+      </c>
+      <c r="F8" t="str">
+        <v>No</v>
+      </c>
+      <c r="I8" t="str">
         <v>https://1fichier.com/?njtt4tcu804msjd3gyyo</v>
       </c>
-      <c r="L8" t="str">
+      <c r="M8" t="str">
         <v>https://megaup.net/8104a051efe3cef06e7baac9b73da32c/SubZero.rar</v>
       </c>
-      <c r="M8" t="str">
+      <c r="N8" t="str">
         <v>https://gofile.io/d/0IrgTE</v>
       </c>
-      <c r="N8" t="str">
+      <c r="O8" t="str">
         <v>https://downloadgameps3.net/archives/18667</v>
       </c>
     </row>
@@ -717,24 +742,27 @@
         <v>imagenes/PC/Touhou Erosion The Fallen Shrine Maiden of Paradis.jpg</v>
       </c>
       <c r="E9" t="str">
-        <v>No</v>
+        <v>No disponible</v>
       </c>
       <c r="F9" t="str">
+        <v>No</v>
+      </c>
+      <c r="G9" t="str">
         <v>https://mega.nz/file/sqA1hKTJ#fbBUIf3xkVaJHKRpm37GgEbgNrk8RY6ZmqU8kUAGYUo</v>
       </c>
-      <c r="H9" t="str">
+      <c r="I9" t="str">
         <v>https://1fichier.com/?z5cue67si7l1hfq7dsmq</v>
       </c>
-      <c r="L9" t="str">
+      <c r="M9" t="str">
         <v>https://megaup.net/830c41ed74360deab38ea08d8fef1597/Touhou.Erosion.The.Fallen.Shrine.Maiden.of.Paradise-TENOKE.rar</v>
       </c>
-      <c r="M9" t="str">
+      <c r="N9" t="str">
         <v>https://send.now/d/1lMeL</v>
       </c>
-      <c r="N9" t="str">
+      <c r="O9" t="str">
         <v>https://gofile.io/d/xba3UN</v>
       </c>
-      <c r="O9" t="str">
+      <c r="P9" t="str">
         <v>https://downloadgameps3.net/archives/18667</v>
       </c>
     </row>
@@ -752,24 +780,27 @@
         <v>imagenes/PC/Solarpunk.jpg</v>
       </c>
       <c r="E10" t="str">
-        <v>No</v>
+        <v>No disponible</v>
       </c>
       <c r="F10" t="str">
+        <v>No</v>
+      </c>
+      <c r="G10" t="str">
         <v>https://mega.nz/file/CpYjgZiR#AmWM1KvAFtFHDXi0pMIAihUcbqXPYFg9ppxjB4X_Ev8</v>
       </c>
-      <c r="H10" t="str">
+      <c r="I10" t="str">
         <v>https://1fichier.com/?p23pohmy9e16829ysvqs</v>
       </c>
-      <c r="L10" t="str">
+      <c r="M10" t="str">
         <v>https://megaup.net/f4d996f43210497b1d734a40cc071f5d/Solarpunk.rar</v>
       </c>
-      <c r="M10" t="str">
+      <c r="N10" t="str">
         <v>https://send.now/hdemjtxgx55j</v>
       </c>
-      <c r="N10" t="str">
+      <c r="O10" t="str">
         <v>https://gofile.io/d/sQ7KbV</v>
       </c>
-      <c r="O10" t="str">
+      <c r="P10" t="str">
         <v>https://downloadgameps3.net/archives/18667</v>
       </c>
     </row>
@@ -787,24 +818,27 @@
         <v>imagenes/PC/Terrinoth Heroes of Descent.jpg</v>
       </c>
       <c r="E11" t="str">
-        <v>No</v>
+        <v>No disponible</v>
       </c>
       <c r="F11" t="str">
+        <v>No</v>
+      </c>
+      <c r="G11" t="str">
         <v>https://mega.nz/file/HoxUHZyC#Ss7RZoQlKLGmTkVkwIft4_BG2g5X3Y3ep7BhlQyYr6M</v>
       </c>
-      <c r="H11" t="str">
+      <c r="I11" t="str">
         <v>https://1fichier.com/?1ufhqw3hkjz3t3947pgm</v>
       </c>
-      <c r="L11" t="str">
+      <c r="M11" t="str">
         <v>https://megaup.net/d2ab5b0981758764f4983fed57c9c357/Terrinoth.Heroes.of.Descent.rar</v>
       </c>
-      <c r="M11" t="str">
+      <c r="N11" t="str">
         <v>https://send.now/h6sld2d7x54d</v>
       </c>
-      <c r="N11" t="str">
+      <c r="O11" t="str">
         <v>https://gofile.io/d/Rgxgp2</v>
       </c>
-      <c r="O11" t="str">
+      <c r="P11" t="str">
         <v>https://downloadgameps3.net/archives/18667</v>
       </c>
     </row>
@@ -822,24 +856,27 @@
         <v>imagenes/PC/Exo Rally Championship.jpg</v>
       </c>
       <c r="E12" t="str">
-        <v>No</v>
+        <v>No disponible</v>
       </c>
       <c r="F12" t="str">
+        <v>No</v>
+      </c>
+      <c r="G12" t="str">
         <v>https://mega.nz/file/n4gS2AiB#u4B4RCzi2MbwiZMlyhpQQcAciglm1A3mqyVKQU7Vgl8</v>
       </c>
-      <c r="H12" t="str">
+      <c r="I12" t="str">
         <v>https://1fichier.com/?u470w1glmhrqms1rqhzt</v>
       </c>
-      <c r="L12" t="str">
+      <c r="M12" t="str">
         <v>https://megaup.net/9c5afca9d7f99967a063f3c6de3c04a3/Exo.Rally.Championship.rar</v>
       </c>
-      <c r="M12" t="str">
+      <c r="N12" t="str">
         <v>https://send.now/d/1lJzY</v>
       </c>
-      <c r="N12" t="str">
+      <c r="O12" t="str">
         <v>https://gofile.io/d/VzbBqn</v>
       </c>
-      <c r="O12" t="str">
+      <c r="P12" t="str">
         <v>https://downloadgameps3.net/archives/18667</v>
       </c>
     </row>
@@ -857,24 +894,27 @@
         <v>imagenes/PC/Momento.jpg</v>
       </c>
       <c r="E13" t="str">
-        <v>No</v>
+        <v>No disponible</v>
       </c>
       <c r="F13" t="str">
+        <v>No</v>
+      </c>
+      <c r="G13" t="str">
         <v>https://mega.nz/file/GO5zUYjD#plSYvTIkXIq2d09CNQmGQfVbaWKbV92JqwGGjCGaaG4</v>
       </c>
-      <c r="H13" t="str">
+      <c r="I13" t="str">
         <v>https://1fichier.com/?5eclk743q2dnkv17cy1l</v>
       </c>
-      <c r="L13" t="str">
+      <c r="M13" t="str">
         <v>https://megaup.net/413b8f61b6686136b8e6d1e5d223ed3b/Momento.rar</v>
       </c>
-      <c r="M13" t="str">
+      <c r="N13" t="str">
         <v>https://send.now/uvxr8vcg2mfl</v>
       </c>
-      <c r="N13" t="str">
+      <c r="O13" t="str">
         <v>https://gofile.io/d/Zzjd5C</v>
       </c>
-      <c r="O13" t="str">
+      <c r="P13" t="str">
         <v>https://downloadgameps3.net/archives/18667</v>
       </c>
     </row>
@@ -892,24 +932,27 @@
         <v>imagenes/PC/OddFauna Secret of the Terrabeast.jpg</v>
       </c>
       <c r="E14" t="str">
-        <v>No</v>
+        <v>No disponible</v>
       </c>
       <c r="F14" t="str">
+        <v>No</v>
+      </c>
+      <c r="G14" t="str">
         <v>https://mega.nz/file/TgRVAJYT#8dQQ_r0QzQe2IaEVs-kQBYfthB0QMxApGRl8xf5rj_Q</v>
       </c>
-      <c r="H14" t="str">
+      <c r="I14" t="str">
         <v>https://1fichier.com/?bfu4thgtcy38gn0gxj5b</v>
       </c>
-      <c r="L14" t="str">
+      <c r="M14" t="str">
         <v>https://megaup.net/d179aa4d9cc5e1867cbdb178d40a08c1/OddFauna.Secret.of.the.Terrabeast.rar</v>
       </c>
-      <c r="M14" t="str">
+      <c r="N14" t="str">
         <v>https://send.now/d/1lM4C</v>
       </c>
-      <c r="N14" t="str">
+      <c r="O14" t="str">
         <v>https://gofile.io/d/ujmexR</v>
       </c>
-      <c r="O14" t="str">
+      <c r="P14" t="str">
         <v>https://downloadgameps3.net/archives/18667</v>
       </c>
     </row>
@@ -927,24 +970,27 @@
         <v>imagenes/PC/Trading Card Inspector.jpg</v>
       </c>
       <c r="E15" t="str">
-        <v>No</v>
+        <v>No disponible</v>
       </c>
       <c r="F15" t="str">
+        <v>No</v>
+      </c>
+      <c r="G15" t="str">
         <v>https://mega.nz/file/rgAEQADZ#kZ8a_g_wr_X4Hy6Zvrnh-awGaJE45YQ33UixGLjjshY</v>
       </c>
-      <c r="H15" t="str">
+      <c r="I15" t="str">
         <v>https://1fichier.com/?aq6fs8az7oelg5rnbq9d</v>
       </c>
-      <c r="L15" t="str">
+      <c r="M15" t="str">
         <v>https://megaup.net/d90025c15ceacd6bef4798ccbc84739f/Trading.Card.Inspector.rar</v>
       </c>
-      <c r="M15" t="str">
+      <c r="N15" t="str">
         <v>https://send.now/d/1lM0f</v>
       </c>
-      <c r="N15" t="str">
+      <c r="O15" t="str">
         <v>https://gofile.io/d/iF0vqe</v>
       </c>
-      <c r="O15" t="str">
+      <c r="P15" t="str">
         <v>https://downloadgameps3.net/archives/18667</v>
       </c>
     </row>
@@ -962,24 +1008,27 @@
         <v>imagenes/PC/Your Own Cozy Motel.jpg</v>
       </c>
       <c r="E16" t="str">
-        <v>No</v>
+        <v>No disponible</v>
       </c>
       <c r="F16" t="str">
+        <v>No</v>
+      </c>
+      <c r="G16" t="str">
         <v>https://mega.nz/file/akoQRKiT#w1AgnY0jLSIE7N99k1xm_IOgq_UQ5MFK4L0jJqw6nwg</v>
       </c>
-      <c r="H16" t="str">
+      <c r="I16" t="str">
         <v>https://1fichier.com/?o8iirmqivun0x4s7ays2</v>
       </c>
-      <c r="L16" t="str">
+      <c r="M16" t="str">
         <v>https://megaup.net/e385bf9ca47cbe8a593aea0da88f3307/Your.Own.Cozy.Motel.rar</v>
       </c>
-      <c r="M16" t="str">
+      <c r="N16" t="str">
         <v>https://send.now/d/1lM1M</v>
       </c>
-      <c r="N16" t="str">
+      <c r="O16" t="str">
         <v>https://gofile.io/d/5Jyj9f</v>
       </c>
-      <c r="O16" t="str">
+      <c r="P16" t="str">
         <v>https://downloadgameps3.net/archives/18667</v>
       </c>
     </row>
@@ -997,24 +1046,27 @@
         <v>imagenes/PC/Tiny Town Market Simulator.jpg</v>
       </c>
       <c r="E17" t="str">
-        <v>No</v>
+        <v>No disponible</v>
       </c>
       <c r="F17" t="str">
+        <v>No</v>
+      </c>
+      <c r="G17" t="str">
         <v>https://mega.nz/file/G4BjCKLb#2Acr23JK0joBETuExsLpw67jt4_P0z-6ZghmpmHcgBQ</v>
       </c>
-      <c r="H17" t="str">
+      <c r="I17" t="str">
         <v>https://1fichier.com/?mlk2h5s03eofbs4vfp0s</v>
       </c>
-      <c r="L17" t="str">
+      <c r="M17" t="str">
         <v>https://megaup.net/e972edf9258249b14ea92d43293b9f4e/Tiny.Town.Market.Simulator.rar</v>
       </c>
-      <c r="M17" t="str">
+      <c r="N17" t="str">
         <v>https://send.now/d/1lM1D</v>
       </c>
-      <c r="N17" t="str">
+      <c r="O17" t="str">
         <v>https://gofile.io/d/xSo8yr</v>
       </c>
-      <c r="O17" t="str">
+      <c r="P17" t="str">
         <v>https://downloadgameps3.net/archives/18667</v>
       </c>
     </row>
@@ -1032,24 +1084,27 @@
         <v>imagenes/PC/Beaming.jpg</v>
       </c>
       <c r="E18" t="str">
-        <v>No</v>
+        <v>No disponible</v>
       </c>
       <c r="F18" t="str">
+        <v>No</v>
+      </c>
+      <c r="G18" t="str">
         <v>https://mega.nz/file/C04BEbab#H8KLnLEZUWwd0Q_nk1S5drApHVI1Uq6hjUzHWd2ebbQ</v>
       </c>
-      <c r="H18" t="str">
+      <c r="I18" t="str">
         <v>https://1fichier.com/?1s2m2nnqzg2cjs3ts75q</v>
       </c>
-      <c r="L18" t="str">
+      <c r="M18" t="str">
         <v>https://megaup.net/5f163a83a1da35474022b7db34fdbc00/Beaming.rar</v>
       </c>
-      <c r="M18" t="str">
+      <c r="N18" t="str">
         <v>https://send.now/d/1lM2D</v>
       </c>
-      <c r="N18" t="str">
+      <c r="O18" t="str">
         <v>https://gofile.io/d/Lat8ss</v>
       </c>
-      <c r="O18" t="str">
+      <c r="P18" t="str">
         <v>https://downloadgameps3.net/archives/18667</v>
       </c>
     </row>
@@ -1067,24 +1122,27 @@
         <v>imagenes/PC/The Brewline.jpg</v>
       </c>
       <c r="E19" t="str">
-        <v>No</v>
+        <v>No disponible</v>
       </c>
       <c r="F19" t="str">
+        <v>No</v>
+      </c>
+      <c r="G19" t="str">
         <v>https://mega.nz/file/S9ZzRByS#tQdNphUIOVyMto27KjIDCrbxJdpn2N6wl7h4dZDHYdM</v>
       </c>
-      <c r="H19" t="str">
+      <c r="I19" t="str">
         <v>https://1fichier.com/?8hzvvx90b01ruuge7llf</v>
       </c>
-      <c r="L19" t="str">
+      <c r="M19" t="str">
         <v>https://megaup.net/2929c2cb66f30de58dd632f62f7655c9/The.Brewline.rar</v>
       </c>
-      <c r="M19" t="str">
+      <c r="N19" t="str">
         <v>https://send.now/kx6g2halucac</v>
       </c>
-      <c r="N19" t="str">
+      <c r="O19" t="str">
         <v>https://gofile.io/d/4Mkzs1</v>
       </c>
-      <c r="O19" t="str">
+      <c r="P19" t="str">
         <v>https://downloadgameps3.net/archives/18667</v>
       </c>
     </row>
@@ -1102,24 +1160,27 @@
         <v>imagenes/PC/Ice Cream Simulator.jpg</v>
       </c>
       <c r="E20" t="str">
-        <v>No</v>
+        <v>No disponible</v>
       </c>
       <c r="F20" t="str">
+        <v>No</v>
+      </c>
+      <c r="G20" t="str">
         <v>https://mega.nz/file/XexgyA7D#fkJULBVHF2x7SRZ7VGuMP8t0wb9ZFiizC4zYp6UlF4s</v>
       </c>
-      <c r="H20" t="str">
+      <c r="I20" t="str">
         <v>https://1fichier.com/?us5n66e2npch9t7zribz</v>
       </c>
-      <c r="L20" t="str">
+      <c r="M20" t="str">
         <v>https://megaup.net/7028c85143f6d4ca974defbfe4c1b09a/Ice.Cream.Simulator.rar</v>
       </c>
-      <c r="M20" t="str">
+      <c r="N20" t="str">
         <v>https://send.now/d/1lIIM</v>
       </c>
-      <c r="N20" t="str">
+      <c r="O20" t="str">
         <v>https://gofile.io/d/uoUFXM</v>
       </c>
-      <c r="O20" t="str">
+      <c r="P20" t="str">
         <v>https://downloadgameps3.net/archives/18667</v>
       </c>
     </row>
@@ -1137,30 +1198,33 @@
         <v>imagenes/PC/Tattoo Removal Simulator.jpg</v>
       </c>
       <c r="E21" t="str">
-        <v>No</v>
+        <v>No disponible</v>
       </c>
       <c r="F21" t="str">
+        <v>No</v>
+      </c>
+      <c r="G21" t="str">
         <v>https://mega.nz/file/jDgzyZKa#2CLpvukQqUmOmEnt7FtXc8YvvgUPyoNsmpsb8nXbZtA</v>
       </c>
-      <c r="H21" t="str">
+      <c r="I21" t="str">
         <v>https://1fichier.com/?8w40um9wzo24jiiiia28</v>
       </c>
-      <c r="L21" t="str">
+      <c r="M21" t="str">
         <v>https://megaup.net/795a04588a933aace87ae14e1cd28c49/Tattoo.Removal.Simulator.rar</v>
       </c>
-      <c r="M21" t="str">
+      <c r="N21" t="str">
         <v>https://send.now/d/1lIHz</v>
       </c>
-      <c r="N21" t="str">
+      <c r="O21" t="str">
         <v>https://gofile.io/d/H8MAjl</v>
       </c>
-      <c r="O21" t="str">
+      <c r="P21" t="str">
         <v>https://downloadgameps3.net/archives/18667</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q21"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>